<commit_message>
Update test file for sparklines
Sparkline external reference in the file is kept.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Other/Sparklines/SourceDataFormulas/ExternalReference-output.xlsx
+++ b/ClosedXML.Tests/Resource/Other/Sparklines/SourceDataFormulas/ExternalReference-output.xlsx
@@ -80,204 +80,147 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac x16r2">
-  <x:numFmts count="11">
-    <x:numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <x:numFmt numFmtId="164" formatCode="0.0000%"/>
-    <x:numFmt numFmtId="165" formatCode="0.000000"/>
-    <x:numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
-    <x:numFmt numFmtId="167" formatCode="0.000000%"/>
-    <x:numFmt numFmtId="168" formatCode="0.000%"/>
-    <x:numFmt numFmtId="169" formatCode="#,##0.000%"/>
-    <x:numFmt numFmtId="170" formatCode="#,##0.000000%"/>
-    <x:numFmt numFmtId="171" formatCode="#,##0.000"/>
-    <x:numFmt numFmtId="172" formatCode="0.0%"/>
-    <x:numFmt numFmtId="173" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-  </x:numFmts>
-  <x:fonts count="4" x14ac:knownFonts="1">
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-      <x:scheme val="minor"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color theme="1"/>
-      <x:name val="Consolas"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="3">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor theme="0" tint="-4.9989318521683403E-2"/>
-        <x:bgColor indexed="64"/>
-      </x:patternFill>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="21">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
-    <x:xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <x:xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <x:xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="0" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="167" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="168" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="2" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="3" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="1" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="10" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="169" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="170" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="171" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="172" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="173" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="23">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="170" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="171" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <x:xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="5">
-    <x:cellStyle name="Comma 2" xfId="4"/>
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <x:cellStyle name="Normal 2" xfId="2"/>
-    <x:cellStyle name="Percent" xfId="1" builtinId="5"/>
-    <x:cellStyle name="Percent 2" xfId="3"/>
-  </x:cellStyles>
-  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <x:extLst>
-    <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="11">
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0000%"/>
+    <numFmt numFmtId="166" formatCode="0.000000"/>
+    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="168" formatCode="0.000000%"/>
+    <numFmt numFmtId="169" formatCode="0.000%"/>
+    <numFmt numFmtId="170" formatCode="#,##0.000%"/>
+    <numFmt numFmtId="171" formatCode="#,##0.000000%"/>
+    <numFmt numFmtId="172" formatCode="#,##0.000"/>
+    <numFmt numFmtId="173" formatCode="0.0%"/>
+    <numFmt numFmtId="174" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="3">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="3">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.0499893185216834"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="5">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+  </cellStyleXfs>
+  <cellXfs count="22">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+  </cellXfs>
+  <cellStyles count="5">
+    <cellStyle name="Comma 2" xfId="0" customBuiltin="0"/>
+    <cellStyle name="Normal" xfId="1" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" customBuiltin="0"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Percent 2" xfId="4" customBuiltin="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </x:ext>
-    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
       <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </x:ext>
-  </x:extLst>
-</x:styleSheet>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -627,7 +570,7 @@
       </x:c>
     </x:row>
     <x:row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <x:c r="A2" s="22">
+      <x:c r="A2" s="20">
         <x:f>VLOOKUP(TEXT(B2, 0),Sheet2!A:L,12,FALSE)</x:f>
       </x:c>
       <x:c r="B2" s="0">

</xml_diff>